<commit_message>
fix(audit): synchronize spec function names, align v0 latent risk guard statuses, and enhance CWE/ASan evidence
</commit_message>
<xml_diff>
--- a/docs/02_Risk_Scenarios/scenario_matrix.xlsx
+++ b/docs/02_Risk_Scenarios/scenario_matrix.xlsx
@@ -673,7 +673,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>add_product_to_list</t>
+          <t>add_product</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>add_product_to_list, free_product_list, inventory_free</t>
+          <t>add_product, product_list_free, inventory_free</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -797,7 +797,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>find_product_by_id, add_product_to_list</t>
+          <t>find_product_by_id, add_product</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>import_product_stock, export_product_stock, update_stock</t>
+          <t>import_stock, export_stock, update_stock</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">

</xml_diff>